<commit_message>
refactoring the code, separation of concern TODO
</commit_message>
<xml_diff>
--- a/test/pipo_sample1.xlsx
+++ b/test/pipo_sample1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21267" windowHeight="8019"/>
+    <workbookView windowWidth="21267" windowHeight="7299"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="3" r:id="rId1"/>
@@ -1333,13 +1333,13 @@
   <cols>
     <col min="1" max="1" width="10.8828828828829"/>
     <col min="2" max="2" width="15.2792792792793" customWidth="1"/>
-    <col min="3" max="3" width="11.7927927927928" customWidth="1"/>
+    <col min="3" max="3" width="11.7927927927928" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="25.1441441441441" customWidth="1"/>
-    <col min="5" max="5" width="12.8828828828829" customWidth="1"/>
-    <col min="6" max="6" width="19.6576576576577" customWidth="1"/>
-    <col min="7" max="7" width="15.954954954955" customWidth="1"/>
-    <col min="8" max="8" width="14.1801801801802" customWidth="1"/>
-    <col min="9" max="9" width="16.8918918918919" customWidth="1"/>
+    <col min="5" max="5" width="12.8828828828829" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6576576576577" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="15.954954954955" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="14.1801801801802" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="16.8918918918919" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="5.18918918918919" customWidth="1"/>
     <col min="11" max="11" width="22.6486486486486" style="1" customWidth="1"/>
     <col min="12" max="12" width="43.0990990990991" customWidth="1"/>
@@ -1621,10 +1621,10 @@
         <v>32</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="K7" s="8">
-        <v>0.731342592592593</v>
+        <v>0.0416666666666667</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
fixes in bypass-master logic and pipo_clm handler
</commit_message>
<xml_diff>
--- a/test/pipo_sample1.xlsx
+++ b/test/pipo_sample1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21267" windowHeight="7299"/>
+    <workbookView windowWidth="21267" windowHeight="8019"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="3" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="38">
   <si>
     <t>Date</t>
   </si>
@@ -1328,7 +1328,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr defaultColWidth="8.79279279279279" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10.8828828828829"/>
@@ -1583,7 +1583,7 @@
         <v>20</v>
       </c>
       <c r="K6" s="8">
-        <v>0.31349537037037</v>
+        <v>0.583333333333333</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>21</v>
@@ -1621,10 +1621,10 @@
         <v>32</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="K7" s="8">
-        <v>0.0416666666666667</v>
+        <v>0.625</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>24</v>
@@ -1665,7 +1665,7 @@
         <v>23</v>
       </c>
       <c r="K8" s="8">
-        <v>0.731354166666667</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>24</v>
@@ -1706,7 +1706,7 @@
         <v>23</v>
       </c>
       <c r="K9" s="8">
-        <v>0.731365740740741</v>
+        <v>0.708333333333333</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>24</v>
@@ -1720,13 +1720,13 @@
         <v>46113</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E10" t="s">
         <v>16</v>
@@ -1741,13 +1741,13 @@
         <v>4700136269</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="K10" s="8">
-        <v>0.773043981481481</v>
+        <v>0.211099537037037</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>24</v>
@@ -1785,13 +1785,13 @@
         <v>36</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="K11" s="8">
-        <v>0.211099537037037</v>
+        <v>0.749837962962963</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="M11" s="5" t="s">
         <v>22</v>
@@ -1802,13 +1802,13 @@
         <v>46113</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E12" t="s">
         <v>16</v>
@@ -1823,103 +1823,266 @@
         <v>4700136269</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="K12" s="8">
-        <v>0.749837962962963</v>
+        <v>0.208333333333333</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="M12" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="2:13">
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-    </row>
-    <row r="14" spans="2:13">
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-    </row>
-    <row r="15" spans="2:13">
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-    </row>
-    <row r="16" spans="2:13">
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-    </row>
-    <row r="17" spans="2:13">
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-    </row>
-    <row r="18" spans="2:13">
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
+    <row r="13" spans="1:13">
+      <c r="A13" s="4">
+        <v>46113</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" s="6">
+        <v>4700136269</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K13" s="8">
+        <v>0.25</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" s="4">
+        <v>46113</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" s="6">
+        <v>4700136269</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K14" s="8">
+        <v>0.291666666666667</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" s="4">
+        <v>46114</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H15" s="6">
+        <v>4700136269</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K15" s="8">
+        <v>0.916666666666667</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H16" s="6">
+        <v>4700136269</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K16" s="8">
+        <v>0.25</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17" s="4">
+        <v>46114</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H17" s="6">
+        <v>4700136269</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K17" s="8">
+        <v>0.875</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" s="6">
+        <v>4700136269</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K18" s="8">
+        <v>0.208333333333333</v>
+      </c>
+      <c r="L18" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M18" s="5" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="19" spans="2:13">
       <c r="B19" s="5"/>
@@ -1991,20 +2154,6 @@
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
     </row>
-    <row r="24" spans="2:13">
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>